<commit_message>
Update bug report template
</commit_message>
<xml_diff>
--- a/Day 03 - Git GitHub Test Documentation/bug-reports/Bug_Report.xlsx
+++ b/Day 03 - Git GitHub Test Documentation/bug-reports/Bug_Report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/eaebac77f309a14c/Desktop/Linkific-Tasks-main/Day 03 - Git GitHub Test Documentation/bug-reports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_AA55D6AF9043746F660160F64A0256BDBAFDA4A1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E894080B-A271-4339-8897-609335D0B779}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_AA55D6AF9043746F660160F64A0256BDBAFDA4A1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A88DDF10-A1CB-417B-A86D-7467CAD2362A}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,9 +34,6 @@
     <t>Module</t>
   </si>
   <si>
-    <t>Environment</t>
-  </si>
-  <si>
     <t>Precondition</t>
   </si>
   <si>
@@ -59,6 +56,9 @@
   </si>
   <si>
     <t>Status</t>
+  </si>
+  <si>
+    <t>Environment Set Up</t>
   </si>
 </sst>
 </file>
@@ -137,6 +137,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -450,31 +454,31 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.35">

</xml_diff>